<commit_message>
wip: chart setter fixes + examples regeneration
</commit_message>
<xml_diff>
--- a/examples/excel/cell-formatting.xlsx
+++ b/examples/excel/cell-formatting.xlsx
@@ -3,11 +3,11 @@
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="rId1"/>
-    <x:sheet name="Fills" sheetId="2" r:id="R423637b7f6014b8d"/>
-    <x:sheet name="Borders" sheetId="3" r:id="Rbb98f24d82534ca6"/>
-    <x:sheet name="Numbers" sheetId="4" r:id="R698bfdc85f8448f5"/>
-    <x:sheet name="Data" sheetId="5" r:id="Rbf7cc62c47cb4ea8"/>
-    <x:sheet name="RichText" sheetId="6" r:id="R2321056e0a034eb5"/>
+    <x:sheet name="Fills" sheetId="2" r:id="Raf72d2b200864da6"/>
+    <x:sheet name="Borders" sheetId="3" r:id="Rbe9d96da87ac4c25"/>
+    <x:sheet name="Numbers" sheetId="4" r:id="R857866ff2b2441d7"/>
+    <x:sheet name="Data" sheetId="5" r:id="Re83252c2e1f24acc"/>
+    <x:sheet name="RichText" sheetId="6" r:id="Re7defb62758c4817"/>
   </x:sheets>
   <x:calcPr fullCalcOnLoad="1"/>
 </x:workbook>
@@ -422,6 +422,115 @@
 </x:styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+        </a:ln>
+        <a:ln w="12700" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+        </a:ln>
+        <a:ln w="19050" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:cols>
@@ -823,7 +932,7 @@
     <x:mergeCell ref="A13:C13"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="Ra6f3ae9e7270429a" tooltip="Open the repo"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="Ra524a1cf945f41b5" tooltip="Open the repo"/>
   </x:hyperlinks>
 </x:worksheet>
 </file>

</xml_diff>